<commit_message>
A 'Portable' column has been added to both indoor and outdoor plants Excel sheets
</commit_message>
<xml_diff>
--- a/data/Indoor plants.xlsx
+++ b/data/Indoor plants.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\landscapingUOB-api\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480F4E72-767D-4FC1-AF70-593AD41BF7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6B233E0-39C5-4F5A-8B4F-EF2CB56FC556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="348">
   <si>
     <t>Plant ID</t>
   </si>
@@ -1075,6 +1075,15 @@
   </si>
   <si>
     <t>Rosa hybrida</t>
+  </si>
+  <si>
+    <t>Portable</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
@@ -2420,7 +2429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I100"/>
+  <dimension ref="A1:J100"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.90625" style="9"/>
@@ -2435,7 +2444,7 @@
     <col min="10" max="16384" width="8.90625" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="7" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" s="7" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -2463,8 +2472,11 @@
       <c r="I1" s="7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" s="7" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J1" s="7" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" s="7" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>9</v>
       </c>
@@ -2493,8 +2505,11 @@
       <c r="I2" s="28" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J2" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>16</v>
       </c>
@@ -2523,8 +2538,11 @@
       <c r="I3" s="28" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J3" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>21</v>
       </c>
@@ -2553,8 +2571,11 @@
       <c r="I4" s="28" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J4" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
         <v>26</v>
       </c>
@@ -2583,8 +2604,11 @@
       <c r="I5" s="28" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J5" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>30</v>
       </c>
@@ -2613,8 +2637,11 @@
       <c r="I6" s="28" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J6" s="7" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
         <v>35</v>
       </c>
@@ -2643,8 +2670,11 @@
       <c r="I7" s="28" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J7" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
         <v>40</v>
       </c>
@@ -2673,8 +2703,11 @@
       <c r="I8" s="28" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J8" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>45</v>
       </c>
@@ -2703,8 +2736,11 @@
       <c r="I9" s="28" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J9" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>49</v>
       </c>
@@ -2733,8 +2769,11 @@
       <c r="I10" s="28" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J10" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>53</v>
       </c>
@@ -2763,8 +2802,11 @@
       <c r="I11" s="28" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J11" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
         <v>58</v>
       </c>
@@ -2793,8 +2835,11 @@
       <c r="I12" s="28" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J12" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
         <v>63</v>
       </c>
@@ -2823,8 +2868,11 @@
       <c r="I13" s="28" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J13" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
         <v>67</v>
       </c>
@@ -2853,8 +2901,11 @@
       <c r="I14" s="28" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J14" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
         <v>72</v>
       </c>
@@ -2883,8 +2934,11 @@
       <c r="I15" s="28" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J15" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
         <v>77</v>
       </c>
@@ -2913,8 +2967,11 @@
       <c r="I16" s="28" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J16" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
         <v>81</v>
       </c>
@@ -2943,8 +3000,11 @@
       <c r="I17" s="28" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J17" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
         <v>85</v>
       </c>
@@ -2973,8 +3033,11 @@
       <c r="I18" s="28" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J18" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
         <v>90</v>
       </c>
@@ -3003,8 +3066,11 @@
       <c r="I19" s="28" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J19" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A20" s="8" t="s">
         <v>95</v>
       </c>
@@ -3033,8 +3099,11 @@
       <c r="I20" s="28" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J20" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
         <v>99</v>
       </c>
@@ -3063,8 +3132,11 @@
       <c r="I21" s="28" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J21" s="7" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
         <v>105</v>
       </c>
@@ -3093,8 +3165,11 @@
       <c r="I22" s="28" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J22" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A23" s="8" t="s">
         <v>109</v>
       </c>
@@ -3123,8 +3198,11 @@
       <c r="I23" s="28" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J23" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A24" s="8" t="s">
         <v>112</v>
       </c>
@@ -3153,8 +3231,11 @@
       <c r="I24" s="28" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J24" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="8" t="s">
         <v>116</v>
       </c>
@@ -3183,8 +3264,11 @@
       <c r="I25" s="28" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J25" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
         <v>120</v>
       </c>
@@ -3213,8 +3297,11 @@
       <c r="I26" s="28" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J26" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="8" t="s">
         <v>124</v>
       </c>
@@ -3243,8 +3330,11 @@
       <c r="I27" s="28" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J27" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A28" s="8" t="s">
         <v>128</v>
       </c>
@@ -3273,8 +3363,11 @@
       <c r="I28" s="28" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J28" s="7" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="s">
         <v>132</v>
       </c>
@@ -3303,8 +3396,11 @@
       <c r="I29" s="28" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J29" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
         <v>137</v>
       </c>
@@ -3333,8 +3429,11 @@
       <c r="I30" s="28" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J30" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A31" s="8" t="s">
         <v>141</v>
       </c>
@@ -3363,8 +3462,11 @@
       <c r="I31" s="28" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J31" s="7" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A32" s="8" t="s">
         <v>145</v>
       </c>
@@ -3393,8 +3495,11 @@
       <c r="I32" s="28" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J32" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A33" s="8" t="s">
         <v>149</v>
       </c>
@@ -3423,8 +3528,11 @@
       <c r="I33" s="28" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J33" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A34" s="8" t="s">
         <v>152</v>
       </c>
@@ -3453,8 +3561,11 @@
       <c r="I34" s="28" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J34" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A35" s="8" t="s">
         <v>156</v>
       </c>
@@ -3483,8 +3594,11 @@
       <c r="I35" s="28" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J35" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="8" t="s">
         <v>160</v>
       </c>
@@ -3513,8 +3627,11 @@
       <c r="I36" s="28" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J36" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A37" s="8" t="s">
         <v>165</v>
       </c>
@@ -3543,8 +3660,11 @@
       <c r="I37" s="28" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J37" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
         <v>170</v>
       </c>
@@ -3573,8 +3693,11 @@
       <c r="I38" s="28" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J38" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A39" s="8" t="s">
         <v>174</v>
       </c>
@@ -3603,8 +3726,11 @@
       <c r="I39" s="28" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J39" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="8" t="s">
         <v>179</v>
       </c>
@@ -3633,8 +3759,11 @@
       <c r="I40" s="28" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J40" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A41" s="8" t="s">
         <v>183</v>
       </c>
@@ -3663,8 +3792,11 @@
       <c r="I41" s="28" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J41" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A42" s="8" t="s">
         <v>187</v>
       </c>
@@ -3693,8 +3825,11 @@
       <c r="I42" s="28" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J42" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A43" s="8" t="s">
         <v>191</v>
       </c>
@@ -3723,8 +3858,11 @@
       <c r="I43" s="28" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J43" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A44" s="8" t="s">
         <v>195</v>
       </c>
@@ -3753,8 +3891,11 @@
       <c r="I44" s="28" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J44" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A45" s="8" t="s">
         <v>199</v>
       </c>
@@ -3783,8 +3924,11 @@
       <c r="I45" s="28" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J45" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A46" s="8" t="s">
         <v>203</v>
       </c>
@@ -3813,8 +3957,11 @@
       <c r="I46" s="28" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J46" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A47" s="8" t="s">
         <v>207</v>
       </c>
@@ -3843,8 +3990,11 @@
       <c r="I47" s="28" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J47" s="7" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A48" s="8" t="s">
         <v>211</v>
       </c>
@@ -3873,8 +4023,11 @@
       <c r="I48" s="28" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J48" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A49" s="8" t="s">
         <v>215</v>
       </c>
@@ -3903,8 +4056,11 @@
       <c r="I49" s="28" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J49" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A50" s="8" t="s">
         <v>219</v>
       </c>
@@ -3933,8 +4089,11 @@
       <c r="I50" s="28" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J50" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A51" s="8" t="s">
         <v>223</v>
       </c>
@@ -3963,8 +4122,11 @@
       <c r="I51" s="28" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J51" s="7" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A52" s="8" t="s">
         <v>227</v>
       </c>
@@ -3993,8 +4155,11 @@
       <c r="I52" s="28" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J52" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A53" s="8" t="s">
         <v>231</v>
       </c>
@@ -4023,8 +4188,11 @@
       <c r="I53" s="28" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J53" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="8" t="s">
         <v>235</v>
       </c>
@@ -4053,8 +4221,11 @@
       <c r="I54" s="28" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="J54" s="7" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A55" s="8"/>
       <c r="B55" s="22"/>
       <c r="C55" s="22"/>
@@ -4062,31 +4233,31 @@
       <c r="E55" s="13"/>
       <c r="H55" s="22"/>
     </row>
-    <row r="56" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A56" s="8"/>
     </row>
-    <row r="57" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A57" s="8"/>
     </row>
-    <row r="58" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A58" s="8"/>
     </row>
-    <row r="59" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A59" s="8"/>
     </row>
-    <row r="60" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A60" s="8"/>
     </row>
-    <row r="61" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A61" s="8"/>
     </row>
-    <row r="62" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A62" s="8"/>
     </row>
-    <row r="63" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A63" s="8"/>
     </row>
-    <row r="64" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A64" s="8"/>
     </row>
     <row r="65" spans="1:1" ht="15.5" x14ac:dyDescent="0.35">
@@ -4202,11 +4373,14 @@
     <cfRule type="duplicateValues" dxfId="89" priority="91"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B54 B1:B26 B48:B50 B31:B46 B52 B56:B1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="2"/>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G35 G37:G1048576" xr:uid="{84F914E3-C5A8-4843-B3F4-1A37C7AF587E}">
       <formula1>"Low,Medium,High"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576" xr:uid="{B838D36E-2CB4-403F-A2B2-DECB211C9D66}">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -7792,220 +7966,220 @@
     <sortCondition ref="B3:B5"/>
   </sortState>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="88" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="34"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31">
-    <cfRule type="duplicateValues" dxfId="87" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="86" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33">
-    <cfRule type="duplicateValues" dxfId="85" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B37">
-    <cfRule type="duplicateValues" dxfId="84" priority="70"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="70"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B38">
-    <cfRule type="duplicateValues" dxfId="83" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="69"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B39">
-    <cfRule type="duplicateValues" dxfId="82" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B40">
-    <cfRule type="duplicateValues" dxfId="81" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B41">
-    <cfRule type="duplicateValues" dxfId="80" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="50"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="duplicateValues" dxfId="79" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="49"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43">
-    <cfRule type="duplicateValues" dxfId="78" priority="48"/>
-    <cfRule type="duplicateValues" dxfId="77" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="duplicateValues" dxfId="76" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="47"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45">
-    <cfRule type="duplicateValues" dxfId="75" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B46">
-    <cfRule type="duplicateValues" dxfId="74" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B47">
-    <cfRule type="duplicateValues" dxfId="73" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B48">
-    <cfRule type="duplicateValues" dxfId="72" priority="90"/>
-    <cfRule type="duplicateValues" dxfId="71" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="90"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B49">
-    <cfRule type="duplicateValues" dxfId="70" priority="89"/>
-    <cfRule type="duplicateValues" dxfId="69" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="89"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B50">
-    <cfRule type="duplicateValues" dxfId="68" priority="66"/>
-    <cfRule type="duplicateValues" dxfId="67" priority="88"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="66"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="88"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B51">
-    <cfRule type="duplicateValues" dxfId="66" priority="87"/>
-    <cfRule type="duplicateValues" dxfId="65" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="87"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B52">
-    <cfRule type="duplicateValues" dxfId="64" priority="23"/>
-    <cfRule type="duplicateValues" dxfId="63" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="65"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B53">
-    <cfRule type="duplicateValues" dxfId="62" priority="64"/>
-    <cfRule type="duplicateValues" dxfId="61" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B54">
-    <cfRule type="duplicateValues" dxfId="60" priority="63"/>
-    <cfRule type="duplicateValues" dxfId="59" priority="46"/>
-    <cfRule type="duplicateValues" dxfId="58" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="46"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B55">
-    <cfRule type="duplicateValues" dxfId="57" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="62"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B56">
-    <cfRule type="duplicateValues" dxfId="56" priority="45"/>
-    <cfRule type="duplicateValues" dxfId="55" priority="61"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="61"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B57">
-    <cfRule type="duplicateValues" dxfId="54" priority="44"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B58">
-    <cfRule type="duplicateValues" dxfId="52" priority="43"/>
-    <cfRule type="duplicateValues" dxfId="51" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="60"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59">
-    <cfRule type="duplicateValues" dxfId="50" priority="59"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B60">
-    <cfRule type="duplicateValues" dxfId="48" priority="58"/>
-    <cfRule type="duplicateValues" dxfId="47" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B61">
-    <cfRule type="duplicateValues" dxfId="46" priority="86"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="86"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="57"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B62">
-    <cfRule type="duplicateValues" dxfId="44" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B63">
-    <cfRule type="duplicateValues" dxfId="43" priority="39"/>
-    <cfRule type="duplicateValues" dxfId="42" priority="85"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="85"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B64">
-    <cfRule type="duplicateValues" dxfId="41" priority="84"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="56"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="84"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B65">
-    <cfRule type="duplicateValues" dxfId="37" priority="83"/>
-    <cfRule type="duplicateValues" dxfId="36" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B66">
-    <cfRule type="duplicateValues" dxfId="35" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="82"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B67">
-    <cfRule type="duplicateValues" dxfId="34" priority="81"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="81"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B68">
-    <cfRule type="duplicateValues" dxfId="33" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69">
-    <cfRule type="duplicateValues" dxfId="32" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="80"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B70">
-    <cfRule type="duplicateValues" dxfId="31" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="79"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B71">
-    <cfRule type="duplicateValues" dxfId="30" priority="55"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="78"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B72">
-    <cfRule type="duplicateValues" dxfId="28" priority="77"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B75">
-    <cfRule type="duplicateValues" dxfId="27" priority="35"/>
-    <cfRule type="duplicateValues" dxfId="26" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="76"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B82">
-    <cfRule type="duplicateValues" dxfId="25" priority="71"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B88">
-    <cfRule type="duplicateValues" dxfId="24" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B98">
-    <cfRule type="duplicateValues" dxfId="23" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B99">
-    <cfRule type="duplicateValues" dxfId="22" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B112">
-    <cfRule type="duplicateValues" dxfId="21" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B113">
-    <cfRule type="duplicateValues" dxfId="20" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B114">
-    <cfRule type="duplicateValues" dxfId="19" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B115">
-    <cfRule type="duplicateValues" dxfId="18" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B119">
-    <cfRule type="duplicateValues" dxfId="17" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="54"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B120">
-    <cfRule type="duplicateValues" dxfId="16" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B121">
-    <cfRule type="duplicateValues" dxfId="15" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B122">
-    <cfRule type="duplicateValues" dxfId="14" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="51"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B137">
-    <cfRule type="duplicateValues" dxfId="13" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B146">
-    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B147">
-    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B151">
-    <cfRule type="duplicateValues" dxfId="10" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="74"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B152">
-    <cfRule type="duplicateValues" dxfId="9" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="73"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B153">
-    <cfRule type="duplicateValues" dxfId="8" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B156">
-    <cfRule type="duplicateValues" dxfId="7" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B161">
-    <cfRule type="duplicateValues" dxfId="6" priority="8"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B162">
-    <cfRule type="duplicateValues" dxfId="3" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B163">
-    <cfRule type="duplicateValues" dxfId="2" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B164">
-    <cfRule type="duplicateValues" dxfId="1" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1 D161:D1048576 D155 D2:D95 D97:D146" xr:uid="{8270B7E8-CE95-4076-B244-68DB0D08C67D}"/>

</xml_diff>